<commit_message>
change the name of id
</commit_message>
<xml_diff>
--- a/data/before_after_0-300/result.xlsx
+++ b/data/before_after_0-300/result.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lijiajun/Desktop/imperial/SWEG/before_after/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lijiajun/Desktop/imperial/SWEG/nlp_grant_coursework/data/before_after_0-300/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD9562A-A40E-BB46-9BF0-DA24801D0B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E5343D-7A3A-3F47-9486-8DFD689E3002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="200" yWindow="1100" windowWidth="30040" windowHeight="17240" xr2:uid="{80634062-07FB-3D4A-A913-40219497547D}"/>
+    <workbookView xWindow="34080" yWindow="1340" windowWidth="30040" windowHeight="17240" xr2:uid="{80634062-07FB-3D4A-A913-40219497547D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="69">
   <si>
     <t>Final score</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -166,19 +166,6 @@
     <t>IC00220_after</t>
   </si>
   <si>
-    <t>IC00228_before</t>
-  </si>
-  <si>
-    <t>0.2 / 5</t>
-  </si>
-  <si>
-    <t>IC00281_before</t>
-  </si>
-  <si>
-    <t>0.2 / 5</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>IC00106_before</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -194,13 +181,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>IC00107_before</t>
-  </si>
-  <si>
-    <t>0/5</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>IC00114_before</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -214,14 +194,105 @@
     <t>3.9 / 5</t>
   </si>
   <si>
+    <t>4.4/5</t>
+  </si>
+  <si>
+    <t>0.2/5</t>
+  </si>
+  <si>
+    <t>0.2/5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.3/5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4.1/5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3.8/5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4.0/5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.5/5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.5/5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.8/5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.2/5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>IC00128_after</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00300_before</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00300_after</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00303_before</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00303_after</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00312_before</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00312_after</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00315_before</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00315_after</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00316_before</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00316_after</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00323_before</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC00323_after</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -245,6 +316,18 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF111827"/>
+      <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -254,7 +337,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -262,21 +345,182 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7EB"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFE5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7EB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7EB"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFE5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7EB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFE5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7EB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7EB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7EB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7EB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7EB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7EB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7EB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7EB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="58" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="1" xr:uid="{977E7743-B65A-FA47-B567-10E8A7F73A81}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -589,7 +833,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9AAA1D1-B15C-8542-8165-CD38EB584CF0}">
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="29.5" customWidth="1"/>
@@ -602,34 +846,33 @@
     <col min="9" max="9" width="33.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="1"/>
+    <row r="1" spans="1:9" s="1" customFormat="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" s="1" customFormat="1">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -639,26 +882,26 @@
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="1">
         <v>76.7</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="1">
         <v>87.7</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="1">
         <v>90</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="1">
         <v>90</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="1">
         <v>80</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="1">
         <v>76.7</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" s="1" customFormat="1">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -668,26 +911,26 @@
       <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="1">
         <v>89.4</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
         <v>90</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="1">
         <v>97.5</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="1">
         <v>97.5</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="1">
         <v>80</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="1">
         <v>75.5</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" s="1" customFormat="1">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -697,605 +940,867 @@
       <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>73.3</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="1">
         <v>15</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="1">
         <v>63.5</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="1">
         <v>17.5</v>
       </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
+      <c r="H4" s="1">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1">
         <v>56.7</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" s="1" customFormat="1">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>84.4</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="1">
         <v>91.1</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="1">
         <v>82.7</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="1">
         <v>89.4</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="1">
         <v>81.2</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="1">
         <v>73.3</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="1">
         <v>88.9</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
+    <row r="6" spans="1:9" s="1" customFormat="1">
+      <c r="A6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>81</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="1">
         <v>80</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="1">
         <v>94</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="1">
         <v>89.4</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="1">
         <v>72.5</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="1">
         <v>93.3</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="1">
         <v>56.7</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
-      <c r="A7" t="s">
+    <row r="7" spans="1:9" s="1" customFormat="1">
+      <c r="A7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="1">
         <v>92</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="1">
         <v>89.4</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="1">
         <v>99</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="1">
         <v>97.5</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="1">
         <v>88.8</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="1">
         <v>91.7</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="1">
         <v>85.6</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
-      <c r="A8" t="s">
+    <row r="8" spans="1:9" s="1" customFormat="1">
+      <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <v>35.799999999999997</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="1">
         <v>71.7</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="1">
         <v>12.3</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="1">
         <v>61.7</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="1">
         <v>20</v>
       </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
+      <c r="H8" s="1">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1">
         <v>48.9</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
-      <c r="A9" t="s">
+    <row r="9" spans="1:9" s="1" customFormat="1">
+      <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>42.2</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="1">
         <v>76.7</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="1">
         <v>10.6</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="1">
         <v>73.8</v>
       </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9">
+      <c r="G9" s="1">
+        <v>0</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
-      <c r="A10" t="s">
+    <row r="10" spans="1:9" s="1" customFormat="1">
+      <c r="A10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <v>49.4</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="1">
         <v>85</v>
       </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
+      <c r="E10" s="1">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1">
         <v>79.400000000000006</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="1">
         <v>42.5</v>
       </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10">
+      <c r="H10" s="1">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
-      <c r="A11" t="s">
+    <row r="11" spans="1:9" s="1" customFormat="1">
+      <c r="A11" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="1">
         <v>72.3</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="1">
         <v>82.8</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="1">
         <v>56.7</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="1">
         <v>90</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="1">
         <v>50</v>
       </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-      <c r="I11">
+      <c r="H11" s="1">
+        <v>0</v>
+      </c>
+      <c r="I11" s="1">
         <v>82.2</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
-      <c r="A12" t="s">
+    <row r="12" spans="1:9" s="1" customFormat="1">
+      <c r="A12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="1">
         <v>43.1</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="1">
         <v>63.3</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="1">
         <v>23.3</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="1">
         <v>65.599999999999994</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="1">
         <v>7.5</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="1">
         <v>56.7</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="1">
         <v>42.2</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
-      <c r="A13" t="s">
+    <row r="13" spans="1:9" s="1" customFormat="1">
+      <c r="A13" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="1">
         <v>49.8</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="1">
         <v>93.3</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="1">
         <v>4.4000000000000004</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="1">
         <v>88.1</v>
       </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="I13">
+      <c r="G13" s="1">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
         <v>63.3</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
-      <c r="A14" t="s">
+    <row r="14" spans="1:9" s="1" customFormat="1">
+      <c r="A14" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="1">
         <v>84.5</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="1">
         <v>89.4</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="1">
         <v>87</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="1">
         <v>95</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="1">
         <v>80</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="1">
         <v>80</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="1">
         <v>75.5</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
-      <c r="A15" t="s">
+    <row r="15" spans="1:9" s="1" customFormat="1">
+      <c r="A15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="1">
         <v>84.8</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="1">
         <v>89.4</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="1">
         <v>87</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="1">
         <v>97.1</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="1">
         <v>80</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="1">
         <v>80</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="1">
         <v>75.5</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
-      <c r="A16" t="s">
+    <row r="16" spans="1:9" s="1" customFormat="1">
+      <c r="A16" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="1">
+        <v>88.8</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="1">
+        <v>85</v>
+      </c>
+      <c r="E16" s="1">
+        <v>90</v>
+      </c>
+      <c r="F16" s="1">
+        <v>89.6</v>
+      </c>
+      <c r="G16" s="1">
+        <v>85</v>
+      </c>
+      <c r="H16" s="1">
+        <v>100</v>
+      </c>
+      <c r="I16" s="1">
+        <v>83.3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" s="1" customFormat="1">
+      <c r="A17" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" s="1">
+        <v>84.8</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="1">
+        <v>89.4</v>
+      </c>
+      <c r="E17" s="1">
+        <v>84</v>
+      </c>
+      <c r="F17" s="1">
+        <v>95</v>
+      </c>
+      <c r="G17" s="1">
+        <v>92.5</v>
+      </c>
+      <c r="H17" s="1">
+        <v>80</v>
+      </c>
+      <c r="I17" s="1">
+        <v>67.8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" s="1" customFormat="1">
+      <c r="A18" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" s="1">
+        <v>83</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="1">
+        <v>91.7</v>
+      </c>
+      <c r="E18" s="1">
+        <v>74</v>
+      </c>
+      <c r="F18" s="1">
+        <v>89.4</v>
+      </c>
+      <c r="G18" s="1">
+        <v>83.8</v>
+      </c>
+      <c r="H18" s="1">
+        <v>78.3</v>
+      </c>
+      <c r="I18" s="1">
+        <v>81.099999999999994</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" s="1" customFormat="1">
+      <c r="A19" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="1">
+        <v>85</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="1">
+        <v>91.7</v>
+      </c>
+      <c r="E19" s="1">
+        <v>76</v>
+      </c>
+      <c r="F19" s="1">
+        <v>91.9</v>
+      </c>
+      <c r="G19" s="1">
+        <v>83.8</v>
+      </c>
+      <c r="H19" s="1">
+        <v>76.7</v>
+      </c>
+      <c r="I19" s="1">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" s="1" customFormat="1">
+      <c r="A20" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="1">
+        <v>81.2</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="1">
+        <v>84.4</v>
+      </c>
+      <c r="E20" s="1">
+        <v>87</v>
+      </c>
+      <c r="F20" s="1">
+        <v>61.4</v>
+      </c>
+      <c r="G20" s="1">
+        <v>100</v>
+      </c>
+      <c r="H20" s="1">
+        <v>86.7</v>
+      </c>
+      <c r="I20" s="1">
+        <v>67.8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" s="1" customFormat="1">
+      <c r="A21" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="1">
+        <v>86.6</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="1">
+        <v>80</v>
+      </c>
+      <c r="E21" s="1">
+        <v>93</v>
+      </c>
+      <c r="F21" s="1">
+        <v>97.5</v>
+      </c>
+      <c r="G21" s="1">
+        <v>80</v>
+      </c>
+      <c r="H21" s="1">
+        <v>80</v>
+      </c>
+      <c r="I21" s="1">
+        <v>88.9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" s="1" customFormat="1">
+      <c r="A22" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="3">
+        <v>86.4</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D22" s="3">
+        <v>88.3</v>
+      </c>
+      <c r="E22" s="3">
+        <v>86</v>
+      </c>
+      <c r="F22" s="3">
+        <v>90.8</v>
+      </c>
+      <c r="G22" s="3">
+        <v>78.8</v>
+      </c>
+      <c r="H22" s="3">
+        <v>93.3</v>
+      </c>
+      <c r="I22" s="4">
+        <v>81.099999999999994</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" s="1" customFormat="1">
+      <c r="A23" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" s="6">
         <v>8.9</v>
       </c>
-      <c r="C16" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16">
+      <c r="C23" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" s="6">
         <v>53.3</v>
       </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-      <c r="G16">
-        <v>0</v>
-      </c>
-      <c r="H16">
-        <v>0</v>
-      </c>
-      <c r="I16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17" t="s">
-        <v>39</v>
-      </c>
-      <c r="B17">
+      <c r="E23" s="6">
+        <v>0</v>
+      </c>
+      <c r="F23" s="6">
+        <v>0</v>
+      </c>
+      <c r="G23" s="6">
+        <v>0</v>
+      </c>
+      <c r="H23" s="6">
+        <v>0</v>
+      </c>
+      <c r="I23" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" s="1" customFormat="1">
+      <c r="A24" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" s="6">
+        <v>49.8</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D24" s="6">
+        <v>80</v>
+      </c>
+      <c r="E24" s="6">
+        <v>13.3</v>
+      </c>
+      <c r="F24" s="6">
+        <v>66.7</v>
+      </c>
+      <c r="G24" s="6">
+        <v>62.5</v>
+      </c>
+      <c r="H24" s="6">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="I24" s="7">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" s="1" customFormat="1">
+      <c r="A25" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B25" s="6">
         <v>7.8</v>
       </c>
-      <c r="C17" t="s">
-        <v>40</v>
-      </c>
-      <c r="D17">
+      <c r="C25" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" s="6">
         <v>46.7</v>
       </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="H17">
-        <v>0</v>
-      </c>
-      <c r="I17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18">
-        <v>88.8</v>
-      </c>
-      <c r="C18" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18">
+      <c r="E25" s="6">
+        <v>0</v>
+      </c>
+      <c r="F25" s="6">
+        <v>0</v>
+      </c>
+      <c r="G25" s="6">
+        <v>0</v>
+      </c>
+      <c r="H25" s="6">
+        <v>0</v>
+      </c>
+      <c r="I25" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" s="1" customFormat="1">
+      <c r="A26" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B26" s="6">
+        <v>32.4</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" s="6">
+        <v>78.3</v>
+      </c>
+      <c r="E26" s="6">
+        <v>18.3</v>
+      </c>
+      <c r="F26" s="6">
+        <v>65.8</v>
+      </c>
+      <c r="G26" s="6">
+        <v>0</v>
+      </c>
+      <c r="H26" s="6">
+        <v>0</v>
+      </c>
+      <c r="I26" s="7">
+        <v>32.200000000000003</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" s="1" customFormat="1">
+      <c r="A27" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B27" s="6">
+        <v>43.5</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" s="6">
+        <v>76.7</v>
+      </c>
+      <c r="E27" s="6">
+        <v>12.2</v>
+      </c>
+      <c r="F27" s="6">
+        <v>87.5</v>
+      </c>
+      <c r="G27" s="6">
+        <v>0</v>
+      </c>
+      <c r="H27" s="6">
+        <v>0</v>
+      </c>
+      <c r="I27" s="7">
+        <v>41.1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" s="1" customFormat="1">
+      <c r="A28" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="6">
+        <v>79.099999999999994</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D28" s="6">
+        <v>73.3</v>
+      </c>
+      <c r="E28" s="6">
+        <v>90</v>
+      </c>
+      <c r="F28" s="6">
+        <v>42.5</v>
+      </c>
+      <c r="G28" s="6">
         <v>85</v>
       </c>
-      <c r="E18">
-        <v>90</v>
-      </c>
-      <c r="F18">
-        <v>89.6</v>
-      </c>
-      <c r="G18">
+      <c r="H28" s="6">
+        <v>91.7</v>
+      </c>
+      <c r="I28" s="7">
+        <v>92.2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" s="1" customFormat="1">
+      <c r="A29" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="6">
+        <v>12.8</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D29" s="6">
+        <v>57.2</v>
+      </c>
+      <c r="E29" s="6">
+        <v>0</v>
+      </c>
+      <c r="F29" s="6">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="G29" s="6">
+        <v>11.2</v>
+      </c>
+      <c r="H29" s="6">
+        <v>0</v>
+      </c>
+      <c r="I29" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" s="1" customFormat="1">
+      <c r="A30" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B30" s="6">
+        <v>45.7</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D30" s="6">
+        <v>73.3</v>
+      </c>
+      <c r="E30" s="6">
+        <v>24</v>
+      </c>
+      <c r="F30" s="6">
+        <v>74.599999999999994</v>
+      </c>
+      <c r="G30" s="6">
+        <v>38.799999999999997</v>
+      </c>
+      <c r="H30" s="6">
+        <v>0</v>
+      </c>
+      <c r="I30" s="7">
+        <v>63.3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" s="1" customFormat="1">
+      <c r="A31" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31" s="6">
+        <v>54.3</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" s="6">
         <v>85</v>
       </c>
-      <c r="H18">
-        <v>100</v>
-      </c>
-      <c r="I18">
-        <v>83.3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19">
-        <v>84.8</v>
-      </c>
-      <c r="C19" t="s">
-        <v>44</v>
-      </c>
-      <c r="D19">
-        <v>89.4</v>
-      </c>
-      <c r="E19">
-        <v>84</v>
-      </c>
-      <c r="F19">
-        <v>95</v>
-      </c>
-      <c r="G19">
-        <v>92.5</v>
-      </c>
-      <c r="H19">
+      <c r="E31" s="6">
+        <v>45.7</v>
+      </c>
+      <c r="F31" s="6">
+        <v>60.4</v>
+      </c>
+      <c r="G31" s="6">
+        <v>52.5</v>
+      </c>
+      <c r="H31" s="6">
+        <v>0</v>
+      </c>
+      <c r="I31" s="7">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" s="1" customFormat="1">
+      <c r="A32" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B32" s="6">
+        <v>49.9</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D32" s="6">
         <v>80</v>
       </c>
-      <c r="I19">
-        <v>67.8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" t="s">
-        <v>45</v>
-      </c>
-      <c r="B20">
-        <v>0</v>
-      </c>
-      <c r="C20" t="s">
-        <v>46</v>
-      </c>
-      <c r="D20">
-        <v>0</v>
-      </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-      <c r="G20">
-        <v>0</v>
-      </c>
-      <c r="H20">
-        <v>0</v>
-      </c>
-      <c r="I20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" t="s">
-        <v>47</v>
-      </c>
-      <c r="B21">
-        <v>83</v>
-      </c>
-      <c r="C21" t="s">
-        <v>21</v>
-      </c>
-      <c r="D21">
-        <v>91.7</v>
-      </c>
-      <c r="E21">
-        <v>74</v>
-      </c>
-      <c r="F21">
-        <v>89.4</v>
-      </c>
-      <c r="G21">
-        <v>83.8</v>
-      </c>
-      <c r="H21">
-        <v>78.3</v>
-      </c>
-      <c r="I21">
-        <v>81.099999999999994</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" t="s">
-        <v>48</v>
-      </c>
-      <c r="B22">
-        <v>85</v>
-      </c>
-      <c r="C22" t="s">
-        <v>17</v>
-      </c>
-      <c r="D22">
-        <v>91.7</v>
-      </c>
-      <c r="E22">
-        <v>76</v>
-      </c>
-      <c r="F22">
-        <v>91.9</v>
-      </c>
-      <c r="G22">
-        <v>83.8</v>
-      </c>
-      <c r="H22">
-        <v>76.7</v>
-      </c>
-      <c r="I22">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" t="s">
-        <v>49</v>
-      </c>
-      <c r="B23">
-        <v>81.2</v>
-      </c>
-      <c r="C23" t="s">
-        <v>50</v>
-      </c>
-      <c r="D23">
+      <c r="E32" s="6">
+        <v>15.6</v>
+      </c>
+      <c r="F32" s="6">
+        <v>87.1</v>
+      </c>
+      <c r="G32" s="6">
+        <v>0</v>
+      </c>
+      <c r="H32" s="6">
+        <v>0</v>
+      </c>
+      <c r="I32" s="7">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" s="1" customFormat="1">
+      <c r="A33" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B33" s="9">
+        <v>50.1</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D33" s="9">
         <v>84.4</v>
       </c>
-      <c r="E23">
-        <v>87</v>
-      </c>
-      <c r="F23">
-        <v>61.4</v>
-      </c>
-      <c r="G23">
-        <v>100</v>
-      </c>
-      <c r="H23">
-        <v>86.7</v>
-      </c>
-      <c r="I23">
-        <v>67.8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" t="s">
-        <v>51</v>
-      </c>
-      <c r="B24">
-        <v>86.6</v>
-      </c>
-      <c r="C24" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24">
+      <c r="E33" s="9">
+        <v>13.9</v>
+      </c>
+      <c r="F33" s="9">
         <v>80</v>
       </c>
-      <c r="E24">
-        <v>93</v>
-      </c>
-      <c r="F24">
-        <v>97.5</v>
-      </c>
-      <c r="G24">
-        <v>80</v>
-      </c>
-      <c r="H24">
-        <v>80</v>
-      </c>
-      <c r="I24">
-        <v>88.9</v>
-      </c>
-    </row>
+      <c r="G33" s="9">
+        <v>0</v>
+      </c>
+      <c r="H33" s="9">
+        <v>0</v>
+      </c>
+      <c r="I33" s="10">
+        <v>72.2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" s="1" customFormat="1"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>